<commit_message>
Mejora de los KPI de Dashboard
</commit_message>
<xml_diff>
--- a/documentación/Cálculos aplicación.xlsx
+++ b/documentación/Cálculos aplicación.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/narcismagrinabalcells/Dropbox/1 - OFICINA/1-PROMOCIMA/02-CAPITAL PRIVADO/30 - Desarrollo/Préstamos/Claude Pro/promocima/documentación/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8F9A3E7-F46F-0B47-8789-72756BC480BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD5C8CC6-27F6-5949-A567-B2F49F561007}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3960" yWindow="4660" windowWidth="45780" windowHeight="19700" activeTab="1" xr2:uid="{7DA0983C-EA6B-584E-90AC-C5A5D261DBFA}"/>
+    <workbookView xWindow="30980" yWindow="1860" windowWidth="26260" windowHeight="19700" activeTab="1" xr2:uid="{7DA0983C-EA6B-584E-90AC-C5A5D261DBFA}"/>
   </bookViews>
   <sheets>
     <sheet name="Cálculo pagos" sheetId="1" r:id="rId1"/>
@@ -123,7 +123,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="223">
   <si>
     <t>Préstamo</t>
   </si>
@@ -176,9 +176,6 @@
     <t>Participado</t>
   </si>
   <si>
-    <t>Desplegado</t>
-  </si>
-  <si>
     <t>Activo</t>
   </si>
   <si>
@@ -650,15 +647,6 @@
     <t>KPI 2</t>
   </si>
   <si>
-    <t>Ingr. Anuales op. Activas</t>
-  </si>
-  <si>
-    <t>Ingr. Anuales part. Activas</t>
-  </si>
-  <si>
-    <t>Ingr. Promocima Gestión</t>
-  </si>
-  <si>
     <t>Rentabilidad Activas</t>
   </si>
   <si>
@@ -671,9 +659,6 @@
     <t>Rentabilidad Total Promocima</t>
   </si>
   <si>
-    <t>Ingr. Apert. Promocima (LTM)</t>
-  </si>
-  <si>
     <t>Aperturas LTM</t>
   </si>
   <si>
@@ -695,9 +680,6 @@
     <t>Operaciones Judicializadas</t>
   </si>
   <si>
-    <t>Operaciones Vivas</t>
-  </si>
-  <si>
     <t>Operaciones Al día</t>
   </si>
   <si>
@@ -756,6 +738,60 @@
   </si>
   <si>
     <t>Desplegadas</t>
+  </si>
+  <si>
+    <t>En cruso</t>
+  </si>
+  <si>
+    <t>En curso</t>
+  </si>
+  <si>
+    <t>Ingresos Anuales op. Activas</t>
+  </si>
+  <si>
+    <t>Ingresos Anuales part. Activas</t>
+  </si>
+  <si>
+    <t>Ingresos Promocima Gestión</t>
+  </si>
+  <si>
+    <t>Ingresos Apert. Promocima (Últimos 12 meses)</t>
+  </si>
+  <si>
+    <t>KPI 5</t>
+  </si>
+  <si>
+    <t>Operaciones En curso</t>
+  </si>
+  <si>
+    <t>Rent op activas</t>
+  </si>
+  <si>
+    <t>OJO, el calcula esto</t>
+  </si>
+  <si>
+    <t>Rentabilidad</t>
+  </si>
+  <si>
+    <t>Participadas</t>
+  </si>
+  <si>
+    <t>Rentabil. Partícipes</t>
+  </si>
+  <si>
+    <t>Rent. Part.</t>
+  </si>
+  <si>
+    <t>Rent tot. Promocima</t>
+  </si>
+  <si>
+    <t>Garantías</t>
+  </si>
+  <si>
+    <t>LTV op.activas</t>
+  </si>
+  <si>
+    <t>Garantías participadas</t>
   </si>
 </sst>
 </file>
@@ -1403,7 +1439,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="11" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="169" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -1494,6 +1530,10 @@
     <xf numFmtId="0" fontId="13" fillId="34" borderId="0" xfId="55" applyAlignment="1">
       <alignment horizontal="left" indent="3"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="59" applyFont="1"/>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="50" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="61">
     <cellStyle name="(0.000)" xfId="59" xr:uid="{360A8815-3031-C74A-BE38-C64C70964821}"/>
@@ -1590,55 +1630,7 @@
       <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
     </dxf>
     <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="2" tint="-0.249977111117893"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="d/m/yy"/>
@@ -1733,6 +1725,31 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="2" tint="-0.249977111117893"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1740,7 +1757,70 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="170" formatCode="#,##0.00;\(#,##0.00\);\-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
@@ -1767,26 +1847,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -1962,33 +2022,10 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="d/m/yy"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="d/m/yy"/>
@@ -2014,7 +2051,7 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="19" formatCode="d/m/yy"/>
     </dxf>
     <dxf>
       <font>
@@ -2039,6 +2076,9 @@
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -2164,20 +2204,6 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="0"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="0"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
       <font>
         <strike val="0"/>
         <outline val="0"/>
@@ -2196,6 +2222,20 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="0"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="0"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2242,6 +2282,7 @@
       <sheetName val="Presentación"/>
       <sheetName val="Empresas"/>
       <sheetName val="Total"/>
+      <sheetName val="1 - Operaciones de Capital Priv"/>
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0" refreshError="1"/>
@@ -2256,13 +2297,14 @@
       <sheetData sheetId="9" refreshError="1"/>
       <sheetData sheetId="10" refreshError="1"/>
       <sheetData sheetId="11" refreshError="1"/>
+      <sheetData sheetId="12" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{342347A0-3718-E543-B254-C58300B4DF45}" name="T_Prestamos" displayName="T_Prestamos" ref="B4:AA69" headerRowDxfId="55" totalsRowDxfId="54" headerRowBorderDxfId="52" tableBorderDxfId="53" headerRowCellStyle="Tit. column." dataCellStyle="Edición">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{342347A0-3718-E543-B254-C58300B4DF45}" name="T_Prestamos" displayName="T_Prestamos" ref="B4:AA69" headerRowDxfId="55" totalsRowDxfId="52" headerRowBorderDxfId="54" tableBorderDxfId="53" headerRowCellStyle="Tit. column." dataCellStyle="Edición">
   <autoFilter ref="B4:AA69" xr:uid="{2F063318-58AF-9349-9E1B-C141B74A1BA4}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:X68">
     <sortCondition ref="B4:B68"/>
@@ -2272,7 +2314,7 @@
     <tableColumn id="2" xr3:uid="{A22A9582-3F78-3444-AACF-4471E1FFDC5C}" name="Nombre" dataDxfId="50" dataCellStyle="Edición"/>
     <tableColumn id="3" xr3:uid="{430690D2-E436-4449-8DBA-2EA7376C4A0E}" name="firma préstamo" dataDxfId="49" dataCellStyle="Edición"/>
     <tableColumn id="4" xr3:uid="{19354164-1119-784C-BFE2-EF1329660502}" name="Años" dataDxfId="48" dataCellStyle="Edición"/>
-    <tableColumn id="6" xr3:uid="{0AEA6368-9C54-7C44-9443-451E4CCF609C}" name="Importe" totalsRowFunction="sum" dataDxfId="46" totalsRowDxfId="47" dataCellStyle="Edición"/>
+    <tableColumn id="6" xr3:uid="{0AEA6368-9C54-7C44-9443-451E4CCF609C}" name="Importe" totalsRowFunction="sum" dataDxfId="47" totalsRowDxfId="46" dataCellStyle="Edición"/>
     <tableColumn id="9" xr3:uid="{1C1D1FFD-2175-2A44-950F-9AEFDB228E84}" name="% interés ordinario" dataDxfId="45" dataCellStyle="Edición"/>
     <tableColumn id="8" xr3:uid="{D85EA2BF-985C-6743-8712-E8CD420D8A24}" name="% interés demora" dataDxfId="44" dataCellStyle="Edición">
       <calculatedColumnFormula>T_Prestamos[[#This Row],[% interés ordinario]]+3%</calculatedColumnFormula>
@@ -2284,8 +2326,8 @@
     <tableColumn id="19" xr3:uid="{DE707FAB-D8A7-D84F-8914-C91853AD3AF2}" name="Destinatario" dataDxfId="41" dataCellStyle="Edición"/>
     <tableColumn id="7" xr3:uid="{7FA0C8EB-4119-DE4C-A037-C6C197DEF23B}" name="Tipo préstamo" dataDxfId="40" dataCellStyle="Edición"/>
     <tableColumn id="20" xr3:uid="{0D7B3CEA-4EEA-2C40-9F0A-7DE79BD814AA}" name="Intermediario" dataDxfId="39" dataCellStyle="Edición"/>
-    <tableColumn id="5" xr3:uid="{179D6707-B68F-2349-9208-DBB351CB6163}" name="Situación" dataDxfId="37" totalsRowDxfId="38" dataCellStyle="Edición"/>
-    <tableColumn id="10" xr3:uid="{B8BA322B-B67C-C349-A58E-6B4223742C3F}" name="Fecha cancelación" dataDxfId="35" totalsRowDxfId="36" dataCellStyle="Edición"/>
+    <tableColumn id="5" xr3:uid="{179D6707-B68F-2349-9208-DBB351CB6163}" name="Situación" dataDxfId="38" totalsRowDxfId="37" dataCellStyle="Edición"/>
+    <tableColumn id="10" xr3:uid="{B8BA322B-B67C-C349-A58E-6B4223742C3F}" name="Fecha cancelación" dataDxfId="36" totalsRowDxfId="35" dataCellStyle="Edición"/>
     <tableColumn id="23" xr3:uid="{C7D61326-25BA-8E43-B283-CD4817088D56}" name="Importe retraso" dataDxfId="34" dataCellStyle="Edición"/>
     <tableColumn id="11" xr3:uid="{446EC477-A97D-B142-81DE-7AD62FD68877}" name="Duración" dataDxfId="33" dataCellStyle="Edición">
       <calculatedColumnFormula>IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</calculatedColumnFormula>
@@ -2293,25 +2335,25 @@
     <tableColumn id="15" xr3:uid="{E18FDF52-5CCA-A244-8C21-8C51330F49E8}" name="Meses" dataDxfId="32" dataCellStyle="Edición">
       <calculatedColumnFormula>IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{8C260D29-CFEC-824D-8A2B-9906DA82D88D}" name="Pendiente" dataDxfId="30" totalsRowDxfId="31" dataCellStyle="Edición">
+    <tableColumn id="14" xr3:uid="{8C260D29-CFEC-824D-8A2B-9906DA82D88D}" name="Pendiente" dataDxfId="31" totalsRowDxfId="30" dataCellStyle="Edición">
       <calculatedColumnFormula>IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",0,IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Americano",T_Prestamos[[#This Row],[Importe]],T_Prestamos[[#This Row],[Importe]]+CUMPRINC(G5/12,E5*12,F5,1,R5,0)))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{70806D64-3BD3-3D4E-AA1B-A15F999F8E49}" name="Intereses anuales" dataDxfId="28" totalsRowDxfId="29" dataCellStyle="Edición">
+    <tableColumn id="16" xr3:uid="{70806D64-3BD3-3D4E-AA1B-A15F999F8E49}" name="Intereses anuales" dataDxfId="29" totalsRowDxfId="28" dataCellStyle="Edición">
       <calculatedColumnFormula>IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",0,IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Americano",T_Prestamos[[#This Row],[Pendiente]]*T_Prestamos[[#This Row],[% interés ordinario]],-CUMIPMT(G5/12,E5*12,F5,R5,R5+11,0)))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{07CDA123-8F83-A047-A4DB-C63F0EA8CE98}" name="% apertura" dataDxfId="26" totalsRowDxfId="27" dataCellStyle="Porcentaje"/>
-    <tableColumn id="18" xr3:uid="{B4599963-AA85-C04E-A1EC-3127FACC74D3}" name="Apertura" dataDxfId="24" totalsRowDxfId="25" dataCellStyle="Porcentaje">
+    <tableColumn id="17" xr3:uid="{07CDA123-8F83-A047-A4DB-C63F0EA8CE98}" name="% apertura" dataDxfId="27" totalsRowDxfId="26" dataCellStyle="Porcentaje"/>
+    <tableColumn id="18" xr3:uid="{B4599963-AA85-C04E-A1EC-3127FACC74D3}" name="Apertura" dataDxfId="25" totalsRowDxfId="24" dataCellStyle="Porcentaje">
       <calculatedColumnFormula>T_Prestamos[[#This Row],[% apertura]]*T_Prestamos[[#This Row],[Importe]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{B2D93394-5C72-CC47-B0A0-D13F7A65C563}" name="Observaciones" dataDxfId="22" totalsRowDxfId="23" dataCellStyle="Edición"/>
-    <tableColumn id="13" xr3:uid="{2AF53BD5-D4D9-0E43-B9F5-732512C399EF}" name="Prestatario" dataDxfId="19" totalsRowDxfId="21" dataCellStyle="Edición"/>
-    <tableColumn id="25" xr3:uid="{2764F342-0D51-A243-97BD-2ACC63680DE9}" name="Primera cuota año" dataDxfId="17" totalsRowDxfId="18" dataCellStyle="(0.000)">
+    <tableColumn id="12" xr3:uid="{B2D93394-5C72-CC47-B0A0-D13F7A65C563}" name="Observaciones" dataDxfId="23" totalsRowDxfId="22" dataCellStyle="Edición"/>
+    <tableColumn id="13" xr3:uid="{2AF53BD5-D4D9-0E43-B9F5-732512C399EF}" name="Prestatario" dataDxfId="21" totalsRowDxfId="20" dataCellStyle="Edición"/>
+    <tableColumn id="25" xr3:uid="{2764F342-0D51-A243-97BD-2ACC63680DE9}" name="Primera cuota año" dataDxfId="19" totalsRowDxfId="18" dataCellStyle="(0.000)">
       <calculatedColumnFormula>IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{DC225DEE-536B-2046-9763-FCBA7A65CDE1}" name="Int. Anual" dataDxfId="16" totalsRowDxfId="20" dataCellStyle="(0.000)">
+    <tableColumn id="24" xr3:uid="{DC225DEE-536B-2046-9763-FCBA7A65CDE1}" name="Int. Anual" dataDxfId="17" totalsRowDxfId="16" dataCellStyle="(0.000)">
       <calculatedColumnFormula>IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Americano",T_Prestamos[[#This Row],[Importe]]*T_Prestamos[[#This Row],[% interés ordinario]],-CUMIPMT(T_Prestamos[[#This Row],[% interés ordinario]]/12,T_Prestamos[[#This Row],[Años]]*12,T_Prestamos[[#This Row],[Importe]],T_Prestamos[[#This Row],[Primera cuota año]],T_Prestamos[[#This Row],[Primera cuota año]]+11,0)),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="27" xr3:uid="{D5575888-D678-0B49-A433-DEFC31AAB8CC}" name="Aperturas LTM" dataDxfId="2" totalsRowDxfId="3" dataCellStyle="(0.000)">
+    <tableColumn id="27" xr3:uid="{D5575888-D678-0B49-A433-DEFC31AAB8CC}" name="Aperturas LTM" dataDxfId="15" totalsRowDxfId="14" dataCellStyle="(0.000)">
       <calculatedColumnFormula>IF(T_Prestamos[[#This Row],[firma préstamo]]&gt;DATE(YEAR(TODAY())-1,MONTH(TODAY()),DAY(TODAY())),T_Prestamos[[#This Row],[Importe]]*T_Prestamos[[#This Row],[% apertura]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2331,31 +2373,31 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{12C36D5C-40B6-3343-86C4-7D4D8310643A}" name="T_Participaciones" displayName="T_Participaciones" ref="B3:P35" totalsRowShown="0" headerRowDxfId="15" headerRowCellStyle="Título" dataCellStyle="Edición">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{12C36D5C-40B6-3343-86C4-7D4D8310643A}" name="T_Participaciones" displayName="T_Participaciones" ref="B3:P35" totalsRowShown="0" headerRowDxfId="13" headerRowCellStyle="Título" dataCellStyle="Edición">
   <autoFilter ref="B3:P35" xr:uid="{DECA43A9-5434-2B4E-B882-FAD35E3A0482}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{E8FAB490-82E4-C348-8B00-ACB6468591F5}" name="CC Prestataria" dataDxfId="14" dataCellStyle="Edición"/>
-    <tableColumn id="6" xr3:uid="{4F68BE3E-1CDD-364A-BA37-6DFAA752660C}" name="Prestatario" dataDxfId="6" dataCellStyle="Edición">
+    <tableColumn id="1" xr3:uid="{E8FAB490-82E4-C348-8B00-ACB6468591F5}" name="CC Prestataria" dataDxfId="12" dataCellStyle="Edición"/>
+    <tableColumn id="6" xr3:uid="{4F68BE3E-1CDD-364A-BA37-6DFAA752660C}" name="Prestatario" dataDxfId="11" dataCellStyle="Edición">
       <calculatedColumnFormula>VLOOKUP(T_Participaciones[[#This Row],[CC Prestataria]],T_Prestamos[#Data],2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{288E584D-F35F-6748-9E62-1902B9D707B8}" name="Importe préstamo" dataDxfId="13" dataCellStyle="(0.000)">
+    <tableColumn id="9" xr3:uid="{288E584D-F35F-6748-9E62-1902B9D707B8}" name="Importe préstamo" dataDxfId="10" dataCellStyle="(0.000)">
       <calculatedColumnFormula>SUMIFS([1]!T_Prestamos[Importe],[1]!T_Prestamos[Centro coste],T_Participaciones[[#This Row],[CC Prestataria]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{29E4AA34-7381-D54C-9A0D-8FAC4F28A051}" name="CC CCPP" dataDxfId="12" dataCellStyle="Edición"/>
-    <tableColumn id="2" xr3:uid="{20824E84-3446-6344-92A9-6AC6149367E0}" name="CCPP" dataDxfId="11" dataCellStyle="Edición">
+    <tableColumn id="8" xr3:uid="{29E4AA34-7381-D54C-9A0D-8FAC4F28A051}" name="CC CCPP" dataDxfId="9" dataCellStyle="Edición"/>
+    <tableColumn id="2" xr3:uid="{20824E84-3446-6344-92A9-6AC6149367E0}" name="CCPP" dataDxfId="8" dataCellStyle="Edición">
       <calculatedColumnFormula>VLOOKUP(T_Participaciones[[#This Row],[CC CCPP]],[1]!T_Participes[#Data],2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{6F7D5CC9-0B3A-C747-A933-D8ADD0638ADD}" name="Importe" dataDxfId="10" dataCellStyle="Edición"/>
-    <tableColumn id="7" xr3:uid="{5E2157C4-CADA-8446-B857-C97148260C86}" name="Participación" dataDxfId="9" dataCellStyle="Porcentaje">
+    <tableColumn id="3" xr3:uid="{6F7D5CC9-0B3A-C747-A933-D8ADD0638ADD}" name="Importe" dataDxfId="7" dataCellStyle="Edición"/>
+    <tableColumn id="7" xr3:uid="{5E2157C4-CADA-8446-B857-C97148260C86}" name="Participación" dataDxfId="6" dataCellStyle="Porcentaje">
       <calculatedColumnFormula>T_Participaciones[[#This Row],[Importe]]/T_Participaciones[[#This Row],[Importe préstamo]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{795919F7-FAEF-F54E-ABEE-9B587E71B471}" name="Fecha firma" dataDxfId="8" dataCellStyle="Edición"/>
-    <tableColumn id="5" xr3:uid="{B49B5FD7-0F0E-8D4B-B212-D7B831E90962}" name="Situación" dataDxfId="7" dataCellStyle="Edición"/>
+    <tableColumn id="4" xr3:uid="{795919F7-FAEF-F54E-ABEE-9B587E71B471}" name="Fecha firma" dataDxfId="5" dataCellStyle="Edición"/>
+    <tableColumn id="5" xr3:uid="{B49B5FD7-0F0E-8D4B-B212-D7B831E90962}" name="Situación" dataDxfId="4" dataCellStyle="Edición"/>
     <tableColumn id="10" xr3:uid="{E00EE774-87FB-2F44-BC7B-5FEF2564B75C}" name="% Gestión" dataCellStyle="Edición"/>
-    <tableColumn id="11" xr3:uid="{11E1E265-333B-0E43-8A29-97F3B0A5FB64}" name="Gestión" dataDxfId="5" dataCellStyle="Edición">
+    <tableColumn id="11" xr3:uid="{11E1E265-333B-0E43-8A29-97F3B0A5FB64}" name="Gestión" dataDxfId="3" dataCellStyle="Edición">
       <calculatedColumnFormula>T_Participaciones[[#This Row],[% Gestión]]*T_Participaciones[[#This Row],[Importe]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{07CCA5B9-C529-7D48-BE58-7C63D99EAC31}" name="Intereses" dataDxfId="4" dataCellStyle="(0.000)">
+    <tableColumn id="12" xr3:uid="{07CCA5B9-C529-7D48-BE58-7C63D99EAC31}" name="Intereses" dataDxfId="2" dataCellStyle="(0.000)">
       <calculatedColumnFormula>SUMIFS(T_Prestamos[Int. Anual],T_Prestamos[Centro coste],T_Participaciones[[#This Row],[CC Prestataria]])*T_Participaciones[[#This Row],[Participación]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="14" xr3:uid="{8932CFAB-1DD6-0A44-A0EA-571E860F5FFF}" name="Apertura" dataDxfId="1" dataCellStyle="(0.000)"/>
@@ -2822,12 +2864,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8AACCD2-8E74-5A4A-A3BE-8E1E8DEA11AA}">
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="19.33203125" customWidth="1"/>
     <col min="3" max="3" width="10.83203125" style="11"/>
-    <col min="5" max="5" width="24.33203125" customWidth="1"/>
+    <col min="5" max="5" width="41" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="23" customWidth="1"/>
     <col min="11" max="11" width="25.5" customWidth="1"/>
     <col min="12" max="12" width="11.5" bestFit="1" customWidth="1"/>
@@ -2836,15 +2879,15 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="F1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
-        <v>17</v>
+        <v>206</v>
       </c>
       <c r="C2" s="62">
         <f>F2+G2</f>
@@ -2861,7 +2904,7 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C3" s="62">
         <f ca="1">F3+G3</f>
@@ -2876,7 +2919,7 @@
         <v>58309.060595885305</v>
       </c>
       <c r="K3" s="64" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
@@ -2895,12 +2938,12 @@
         <v>1475000</v>
       </c>
       <c r="K4" s="65" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C5" s="62">
         <f ca="1">F5+G5</f>
@@ -2919,7 +2962,7 @@
         <v>58309.060595885305</v>
       </c>
       <c r="K5" s="66" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
@@ -2927,55 +2970,55 @@
         <v>2026</v>
       </c>
       <c r="B6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F6" s="11">
         <f ca="1">SUMIFS(T_Prestamos[Int. Anual],T_Prestamos[Situación],"Activos")</f>
         <v>289988.82659054629</v>
       </c>
       <c r="K6" s="67" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F7" s="12">
         <f ca="1">F6/F3</f>
         <v>0.11163088759668932</v>
       </c>
       <c r="K7" s="67" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F8" s="11">
         <f>SUM(T_Participaciones[Intereses])</f>
         <v>165758.75</v>
       </c>
       <c r="K8" s="66" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F9" s="12">
         <f>F8/F4</f>
         <v>0.11237881355932203</v>
       </c>
       <c r="K9" s="65" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F10" s="11">
         <f>SUMIFS(T_Participaciones[Gestión],T_Participaciones[Situación],"Activa")</f>
@@ -2984,7 +3027,7 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F11" s="56">
         <f ca="1">F6-F8+F10</f>
@@ -2993,7 +3036,7 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F12" s="12">
         <f ca="1">F11/F5</f>
@@ -3002,7 +3045,7 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="F13" s="56">
         <f ca="1">SUM(T_Prestamos[Aperturas LTM])</f>
@@ -3011,7 +3054,7 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="F14" s="56">
         <f ca="1">SUM(T_Participaciones[Apertura LTM])</f>
@@ -3020,57 +3063,57 @@
     </row>
     <row r="16" spans="1:15" ht="19" x14ac:dyDescent="0.25">
       <c r="B16" s="14" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C16" s="63"/>
       <c r="E16" s="14" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F16" s="14"/>
       <c r="H16" s="14" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="I16" s="14"/>
       <c r="K16" s="14" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="L16" s="14"/>
       <c r="N16" s="14" t="s">
-        <v>193</v>
+        <v>211</v>
       </c>
       <c r="O16" s="14"/>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.2">
-      <c r="B17" t="s">
-        <v>17</v>
-      </c>
-      <c r="C17" s="11">
+      <c r="B17" s="68" t="s">
+        <v>205</v>
+      </c>
+      <c r="C17" s="69">
         <f>C2</f>
         <v>2781010</v>
       </c>
-      <c r="E17" t="s">
-        <v>175</v>
-      </c>
-      <c r="F17" s="56">
+      <c r="E17" s="68" t="s">
+        <v>207</v>
+      </c>
+      <c r="F17" s="70">
         <f ca="1">F6</f>
         <v>289988.82659054629</v>
       </c>
-      <c r="H17" t="s">
-        <v>194</v>
-      </c>
-      <c r="I17">
+      <c r="H17" s="68" t="s">
+        <v>188</v>
+      </c>
+      <c r="I17" s="68">
         <f>COUNT(T_Prestamos[Centro coste])</f>
         <v>65</v>
       </c>
-      <c r="K17" t="s">
-        <v>202</v>
-      </c>
-      <c r="L17" s="56">
+      <c r="K17" s="68" t="s">
+        <v>196</v>
+      </c>
+      <c r="L17" s="70">
         <f>SUMIFS(T_Prestamos[Garantía],T_Prestamos[Situación],"Activos")+SUMIFS(T_Prestamos[Garantía],T_Prestamos[Situación],"Judicializados")</f>
         <v>10924829.727304058</v>
       </c>
       <c r="N17" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="O17" s="56">
         <f ca="1">(SUMIFS(T_Prestamos[Duración],T_Prestamos[Situación],"Activos")+SUMIFS(T_Prestamos[Duración],T_Prestamos[Situación],"Judicializados"))/(COUNTIFS(T_Prestamos[Situación],"Activos")+COUNTIFS(T_Prestamos[Situación],"Judicializados"))</f>
@@ -3079,35 +3122,35 @@
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C18" s="11">
         <f ca="1">F3</f>
         <v>2597747.208086757</v>
       </c>
       <c r="E18" t="s">
-        <v>176</v>
+        <v>208</v>
       </c>
       <c r="F18" s="56">
         <f>F8</f>
         <v>165758.75</v>
       </c>
       <c r="H18" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="I18">
         <f>COUNTIFS(T_Prestamos[Situación],"Cancelados")</f>
         <v>39</v>
       </c>
       <c r="K18" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="L18" s="12">
         <f>C2/L17</f>
         <v>0.25455865852531462</v>
       </c>
       <c r="N18" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="O18" s="11">
         <f ca="1">SUMIFS(T_Prestamos[Duración],T_Prestamos[Situación],"Cancelados")/COUNTIFS(T_Prestamos[Situación],"Cancelados")</f>
@@ -3116,35 +3159,35 @@
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B19" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C19" s="11">
         <f ca="1">G3</f>
         <v>58309.060595885305</v>
       </c>
       <c r="E19" t="s">
-        <v>177</v>
+        <v>209</v>
       </c>
       <c r="F19" s="56">
         <f>F10</f>
         <v>28500</v>
       </c>
       <c r="H19" t="s">
-        <v>190</v>
+        <v>212</v>
       </c>
       <c r="I19">
         <f>I17-I18</f>
         <v>26</v>
       </c>
       <c r="K19" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="L19" s="56">
         <f>SUM(T_Participaciones[Garantía])</f>
         <v>6091055.8913987586</v>
       </c>
       <c r="N19" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="O19" s="11">
         <f ca="1">SUMIFS(T_Prestamos[Duración],T_Prestamos[Situación],"Activos")/COUNTIFS(T_Prestamos[Situación],"Activos")</f>
@@ -3153,35 +3196,35 @@
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C20" s="12">
         <f ca="1">C19/C17</f>
         <v>2.0966864770671556E-2</v>
       </c>
       <c r="E20" t="s">
-        <v>182</v>
+        <v>210</v>
       </c>
       <c r="F20" s="56">
         <f ca="1">F13-F14</f>
         <v>24612.225000000002</v>
       </c>
       <c r="H20" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="I20">
         <f>COUNTIFS(T_Prestamos[Situación],"Judicializados")</f>
         <v>4</v>
       </c>
       <c r="K20" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="L20" s="12">
         <f>F4/L19</f>
         <v>0.24215834270752012</v>
       </c>
       <c r="N20" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="O20" s="11">
         <f ca="1">SUMIFS(T_Prestamos[Duración],T_Prestamos[Situación],"Judicializados")/COUNTIFS(T_Prestamos[Situación],"Judicializados")</f>
@@ -3190,21 +3233,21 @@
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C21" s="11">
         <f>F4</f>
         <v>1475000</v>
       </c>
       <c r="E21" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="F21" s="12">
         <f ca="1">F17/C18</f>
         <v>0.11163088759668932</v>
       </c>
       <c r="H21" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="I21">
         <f>COUNTIFS(T_Prestamos[Situación],"Activos")</f>
@@ -3213,40 +3256,166 @@
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C22" s="11">
         <f>G4</f>
         <v>0</v>
       </c>
       <c r="E22" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="F22" s="12">
         <f>F8/F4</f>
         <v>0.11237881355932203</v>
       </c>
       <c r="H22" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C23" s="11">
         <f>C22/C21</f>
         <v>0</v>
       </c>
       <c r="E23" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="F23" s="12">
         <f ca="1">(F17-F18+F19+F20)/F5</f>
         <v>0.15795390121054098</v>
       </c>
       <c r="H23" t="s">
-        <v>192</v>
+        <v>186</v>
+      </c>
+    </row>
+    <row r="26" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="E26" t="s">
+        <v>206</v>
+      </c>
+      <c r="F26">
+        <v>2672058</v>
+      </c>
+    </row>
+    <row r="27" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="E27" t="s">
+        <v>200</v>
+      </c>
+      <c r="F27">
+        <v>2598162</v>
+      </c>
+    </row>
+    <row r="28" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="E28" t="s">
+        <v>215</v>
+      </c>
+      <c r="F28">
+        <v>289444</v>
+      </c>
+    </row>
+    <row r="29" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="E29" t="s">
+        <v>161</v>
+      </c>
+      <c r="F29">
+        <v>28500</v>
+      </c>
+    </row>
+    <row r="30" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="E30" t="s">
+        <v>40</v>
+      </c>
+      <c r="F30">
+        <v>25612</v>
+      </c>
+    </row>
+    <row r="31" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="E31" t="s">
+        <v>213</v>
+      </c>
+      <c r="F31" s="71">
+        <f>F28/F27</f>
+        <v>0.11140336899700634</v>
+      </c>
+    </row>
+    <row r="32" spans="2:15" x14ac:dyDescent="0.2">
+      <c r="E32" t="s">
+        <v>214</v>
+      </c>
+      <c r="F32" s="71">
+        <f>F28/F26</f>
+        <v>0.10832249898767167</v>
+      </c>
+    </row>
+    <row r="34" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="E34" t="s">
+        <v>216</v>
+      </c>
+      <c r="F34">
+        <v>1475000</v>
+      </c>
+    </row>
+    <row r="35" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="E35" t="s">
+        <v>217</v>
+      </c>
+      <c r="F35">
+        <v>165759</v>
+      </c>
+    </row>
+    <row r="36" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="E36" t="s">
+        <v>218</v>
+      </c>
+      <c r="F36" s="71">
+        <f>F35/F34</f>
+        <v>0.11237898305084745</v>
+      </c>
+    </row>
+    <row r="37" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="E37" t="s">
+        <v>219</v>
+      </c>
+      <c r="F37" s="71">
+        <f>(F28-F35+F29+F30)/(F27-F34)</f>
+        <v>0.15830040546243551</v>
+      </c>
+    </row>
+    <row r="39" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="E39" t="s">
+        <v>220</v>
+      </c>
+      <c r="F39">
+        <v>10003131</v>
+      </c>
+    </row>
+    <row r="40" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="E40" t="s">
+        <v>221</v>
+      </c>
+      <c r="F40" s="12">
+        <f>F26/F39</f>
+        <v>0.26712216405043582</v>
+      </c>
+    </row>
+    <row r="41" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="E41" t="s">
+        <v>222</v>
+      </c>
+      <c r="F41">
+        <v>5371230</v>
+      </c>
+    </row>
+    <row r="42" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="E42" t="s">
+        <v>221</v>
+      </c>
+      <c r="F42" s="12">
+        <f>F34/F41</f>
+        <v>0.27461121568057967</v>
       </c>
     </row>
   </sheetData>
@@ -3377,7 +3546,7 @@
     </row>
     <row r="3" spans="2:29" s="15" customFormat="1" ht="19" x14ac:dyDescent="0.25">
       <c r="B3" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C3" s="14"/>
       <c r="D3" s="14"/>
@@ -3407,82 +3576,82 @@
     </row>
     <row r="4" spans="2:29" s="18" customFormat="1" ht="34" x14ac:dyDescent="0.2">
       <c r="B4" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="D4" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="E4" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="F4" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="G4" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="H4" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="H4" s="16" t="s">
+      <c r="I4" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="J4" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="J4" s="16" t="s">
+      <c r="K4" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="K4" s="16" t="s">
+      <c r="L4" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="L4" s="16" t="s">
+      <c r="M4" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="M4" s="16" t="s">
+      <c r="N4" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="N4" s="16" t="s">
+      <c r="O4" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="O4" s="16" t="s">
+      <c r="P4" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="P4" s="16" t="s">
+      <c r="Q4" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="Q4" s="16" t="s">
+      <c r="R4" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="R4" s="16" t="s">
+      <c r="S4" s="16" t="s">
         <v>38</v>
-      </c>
-      <c r="S4" s="16" t="s">
-        <v>39</v>
       </c>
       <c r="T4" s="16" t="s">
         <v>3</v>
       </c>
       <c r="U4" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="V4" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="V4" s="16" t="s">
+      <c r="W4" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="W4" s="16" t="s">
+      <c r="X4" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="X4" s="16" t="s">
-        <v>43</v>
-      </c>
       <c r="Y4" s="16" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Z4" s="16" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AA4" s="16" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="AB4" s="17"/>
       <c r="AC4" s="17"/>
@@ -3492,7 +3661,7 @@
         <v>2001</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D5" s="20">
         <v>42883</v>
@@ -3515,16 +3684,16 @@
         <v/>
       </c>
       <c r="K5" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L5" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L5" s="19" t="s">
+      <c r="M5" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M5" s="19" t="s">
+      <c r="N5" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N5" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O5" s="20">
         <v>45770</v>
@@ -3573,7 +3742,7 @@
         <v>2002</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D6" s="20">
         <v>43003</v>
@@ -3596,16 +3765,16 @@
         <v/>
       </c>
       <c r="K6" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L6" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L6" s="19" t="s">
+      <c r="M6" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M6" s="19" t="s">
+      <c r="N6" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N6" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O6" s="20">
         <v>43532</v>
@@ -3654,7 +3823,7 @@
         <v>2003</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D7" s="20">
         <v>43041</v>
@@ -3678,16 +3847,16 @@
         <v/>
       </c>
       <c r="K7" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L7" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L7" s="19" t="s">
+      <c r="M7" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M7" s="19" t="s">
+      <c r="N7" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N7" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O7" s="20">
         <v>44542</v>
@@ -3736,7 +3905,7 @@
         <v>2004</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D8" s="30">
         <v>43040</v>
@@ -3761,16 +3930,16 @@
         <v>7.4413049033340589E-2</v>
       </c>
       <c r="K8" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="L8" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="L8" s="28" t="s">
+      <c r="M8" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="M8" s="28" t="s">
-        <v>47</v>
-      </c>
       <c r="N8" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O8" s="30"/>
       <c r="P8" s="30"/>
@@ -3799,7 +3968,7 @@
       </c>
       <c r="W8" s="28"/>
       <c r="X8" s="28" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="Y8" s="41">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -3821,7 +3990,7 @@
         <v>2005</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D9" s="20">
         <v>43054</v>
@@ -3844,16 +4013,16 @@
         <v/>
       </c>
       <c r="K9" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L9" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L9" s="19" t="s">
+      <c r="M9" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M9" s="19" t="s">
+      <c r="N9" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N9" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O9" s="20">
         <v>43496</v>
@@ -3902,7 +4071,7 @@
         <v>2006</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D10" s="20">
         <v>43055</v>
@@ -3925,16 +4094,16 @@
         <v/>
       </c>
       <c r="K10" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L10" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L10" s="19" t="s">
+      <c r="M10" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M10" s="19" t="s">
+      <c r="N10" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N10" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O10" s="20">
         <v>45188</v>
@@ -3983,7 +4152,7 @@
         <v>2007</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D11" s="20">
         <v>43055</v>
@@ -4006,16 +4175,16 @@
         <v/>
       </c>
       <c r="K11" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L11" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L11" s="19" t="s">
+      <c r="M11" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M11" s="19" t="s">
+      <c r="N11" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N11" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O11" s="20">
         <v>43171</v>
@@ -4064,7 +4233,7 @@
         <v>2008</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D12" s="20">
         <v>42797</v>
@@ -4087,16 +4256,16 @@
         <v/>
       </c>
       <c r="K12" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L12" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L12" s="19" t="s">
+      <c r="M12" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M12" s="19" t="s">
+      <c r="N12" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N12" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O12" s="20">
         <v>43090</v>
@@ -4145,7 +4314,7 @@
         <v>2009</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D13" s="20">
         <v>42648</v>
@@ -4168,16 +4337,16 @@
         <v/>
       </c>
       <c r="K13" s="19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="L13" s="19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M13" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="N13" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N13" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O13" s="20">
         <v>43586</v>
@@ -4226,7 +4395,7 @@
         <v>2010</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D14" s="20">
         <v>43151</v>
@@ -4249,16 +4418,16 @@
         <v/>
       </c>
       <c r="K14" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L14" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L14" s="19" t="s">
+      <c r="M14" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M14" s="19" t="s">
+      <c r="N14" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N14" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O14" s="20">
         <v>43742</v>
@@ -4307,7 +4476,7 @@
         <v>2011</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D15" s="20">
         <v>43167</v>
@@ -4330,16 +4499,16 @@
         <v/>
       </c>
       <c r="K15" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L15" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L15" s="19" t="s">
+      <c r="M15" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M15" s="19" t="s">
+      <c r="N15" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N15" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O15" s="20">
         <v>44855</v>
@@ -4388,7 +4557,7 @@
         <v>2012</v>
       </c>
       <c r="C16" s="28" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D16" s="30">
         <v>43168</v>
@@ -4414,16 +4583,16 @@
         <v>0.16198557145638787</v>
       </c>
       <c r="K16" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="L16" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="L16" s="28" t="s">
+      <c r="M16" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="M16" s="28" t="s">
-        <v>47</v>
-      </c>
       <c r="N16" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O16" s="30"/>
       <c r="P16" s="30"/>
@@ -4451,10 +4620,10 @@
         <v>0</v>
       </c>
       <c r="W16" s="28" t="s">
+        <v>62</v>
+      </c>
+      <c r="X16" s="28" t="s">
         <v>63</v>
-      </c>
-      <c r="X16" s="28" t="s">
-        <v>64</v>
       </c>
       <c r="Y16" s="41">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -4476,7 +4645,7 @@
         <v>2013</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D17" s="20">
         <v>42940</v>
@@ -4500,16 +4669,16 @@
         <v/>
       </c>
       <c r="K17" s="19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="L17" s="19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M17" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="N17" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N17" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O17" s="20">
         <v>43650</v>
@@ -4558,7 +4727,7 @@
         <v>2014</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D18" s="20">
         <v>43179</v>
@@ -4581,16 +4750,16 @@
         <v/>
       </c>
       <c r="K18" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L18" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L18" s="19" t="s">
+      <c r="M18" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M18" s="19" t="s">
+      <c r="N18" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N18" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O18" s="20">
         <v>44978</v>
@@ -4642,7 +4811,7 @@
         <v>2015</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D19" s="20">
         <v>43208</v>
@@ -4665,16 +4834,16 @@
         <v/>
       </c>
       <c r="K19" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L19" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L19" s="19" t="s">
+      <c r="M19" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M19" s="19" t="s">
+      <c r="N19" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N19" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O19" s="20">
         <v>43448</v>
@@ -4726,7 +4895,7 @@
         <v>2016</v>
       </c>
       <c r="C20" s="28" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D20" s="30">
         <v>43279</v>
@@ -4752,16 +4921,16 @@
         <v>9.8323889299076483E-2</v>
       </c>
       <c r="K20" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="L20" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="L20" s="28" t="s">
+      <c r="M20" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="M20" s="28" t="s">
-        <v>47</v>
-      </c>
       <c r="N20" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O20" s="30"/>
       <c r="P20" s="30"/>
@@ -4790,7 +4959,7 @@
       </c>
       <c r="W20" s="28"/>
       <c r="X20" s="28" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="Y20" s="41">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -4810,7 +4979,7 @@
         <v>2017</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D21" s="20">
         <v>43208</v>
@@ -4833,16 +5002,16 @@
         <v/>
       </c>
       <c r="K21" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L21" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L21" s="19" t="s">
+      <c r="M21" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M21" s="19" t="s">
+      <c r="N21" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N21" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O21" s="20">
         <v>43448</v>
@@ -4891,7 +5060,7 @@
         <v>2018</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D22" s="20">
         <v>43300</v>
@@ -4914,16 +5083,16 @@
         <v/>
       </c>
       <c r="K22" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L22" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L22" s="19" t="s">
+      <c r="M22" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M22" s="19" t="s">
+      <c r="N22" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N22" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O22" s="20">
         <v>43796</v>
@@ -4972,7 +5141,7 @@
         <v>2019</v>
       </c>
       <c r="C23" s="35" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D23" s="36">
         <v>43319</v>
@@ -4997,16 +5166,16 @@
         <v>0.10104167183022254</v>
       </c>
       <c r="K23" s="38" t="s">
+        <v>44</v>
+      </c>
+      <c r="L23" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="L23" s="35" t="s">
+      <c r="M23" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="M23" s="35" t="s">
-        <v>47</v>
-      </c>
       <c r="N23" s="35" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O23" s="36"/>
       <c r="P23" s="36"/>
@@ -5034,7 +5203,7 @@
         <v>0</v>
       </c>
       <c r="W23" s="35" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="X23" s="35"/>
       <c r="Y23" s="59">
@@ -5055,7 +5224,7 @@
         <v>2020</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D24" s="20">
         <v>43353</v>
@@ -5078,16 +5247,16 @@
         <v/>
       </c>
       <c r="K24" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L24" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L24" s="19" t="s">
+      <c r="M24" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M24" s="19" t="s">
+      <c r="N24" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N24" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O24" s="20">
         <v>43586</v>
@@ -5136,7 +5305,7 @@
         <v>2021</v>
       </c>
       <c r="C25" s="35" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D25" s="36">
         <v>43375</v>
@@ -5161,16 +5330,16 @@
         <v>5.3565712354973524E-2</v>
       </c>
       <c r="K25" s="38" t="s">
+        <v>44</v>
+      </c>
+      <c r="L25" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="L25" s="35" t="s">
+      <c r="M25" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="M25" s="35" t="s">
-        <v>47</v>
-      </c>
       <c r="N25" s="35" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O25" s="36"/>
       <c r="P25" s="36"/>
@@ -5198,7 +5367,7 @@
         <v>0</v>
       </c>
       <c r="W25" s="35" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="X25" s="35"/>
       <c r="Y25" s="59">
@@ -5219,7 +5388,7 @@
         <v>2022</v>
       </c>
       <c r="C26" s="19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D26" s="20">
         <v>43375</v>
@@ -5242,16 +5411,16 @@
         <v/>
       </c>
       <c r="K26" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L26" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L26" s="19" t="s">
+      <c r="M26" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M26" s="19" t="s">
+      <c r="N26" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N26" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O26" s="20">
         <v>43670</v>
@@ -5300,7 +5469,7 @@
         <v>2023</v>
       </c>
       <c r="C27" s="19" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D27" s="20">
         <v>43382</v>
@@ -5323,16 +5492,16 @@
         <v/>
       </c>
       <c r="K27" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L27" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L27" s="19" t="s">
+      <c r="M27" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M27" s="19" t="s">
+      <c r="N27" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N27" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O27" s="20">
         <v>45007</v>
@@ -5381,7 +5550,7 @@
         <v>2024</v>
       </c>
       <c r="C28" s="19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D28" s="20">
         <v>43503</v>
@@ -5404,16 +5573,16 @@
         <v/>
       </c>
       <c r="K28" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L28" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L28" s="19" t="s">
+      <c r="M28" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M28" s="19" t="s">
+      <c r="N28" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N28" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O28" s="20">
         <v>44742</v>
@@ -5464,7 +5633,7 @@
         <v>2025</v>
       </c>
       <c r="C29" s="19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D29" s="20">
         <v>43503</v>
@@ -5487,16 +5656,16 @@
         <v/>
       </c>
       <c r="K29" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L29" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L29" s="19" t="s">
+      <c r="M29" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M29" s="19" t="s">
+      <c r="N29" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N29" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O29" s="20">
         <v>44134</v>
@@ -5545,7 +5714,7 @@
         <v>2026</v>
       </c>
       <c r="C30" s="28" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D30" s="30">
         <v>43524</v>
@@ -5571,16 +5740,16 @@
         <v>0.18022908150762307</v>
       </c>
       <c r="K30" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="L30" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="L30" s="28" t="s">
+      <c r="M30" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="M30" s="28" t="s">
-        <v>47</v>
-      </c>
       <c r="N30" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O30" s="30"/>
       <c r="P30" s="30"/>
@@ -5609,7 +5778,7 @@
       </c>
       <c r="W30" s="28"/>
       <c r="X30" s="28" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="Y30" s="41">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -5629,7 +5798,7 @@
         <v>2027</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D31" s="20">
         <v>43529</v>
@@ -5652,16 +5821,16 @@
         <v/>
       </c>
       <c r="K31" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L31" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L31" s="19" t="s">
+      <c r="M31" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M31" s="19" t="s">
+      <c r="N31" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N31" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O31" s="20">
         <v>43799</v>
@@ -5710,7 +5879,7 @@
         <v>2028</v>
       </c>
       <c r="C32" s="28" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D32" s="30">
         <v>43543</v>
@@ -5736,16 +5905,16 @@
         <v>0.18131931068931431</v>
       </c>
       <c r="K32" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="L32" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="L32" s="28" t="s">
+      <c r="M32" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="M32" s="28" t="s">
-        <v>47</v>
-      </c>
       <c r="N32" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O32" s="30"/>
       <c r="P32" s="30"/>
@@ -5774,7 +5943,7 @@
       </c>
       <c r="W32" s="28"/>
       <c r="X32" s="28" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="Y32" s="41">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -5794,7 +5963,7 @@
         <v>2029</v>
       </c>
       <c r="C33" s="19" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D33" s="20">
         <v>43565</v>
@@ -5817,16 +5986,16 @@
         <v/>
       </c>
       <c r="K33" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L33" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L33" s="19" t="s">
+      <c r="M33" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M33" s="19" t="s">
+      <c r="N33" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N33" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O33" s="20">
         <v>43719</v>
@@ -5875,7 +6044,7 @@
         <v>2030</v>
       </c>
       <c r="C34" s="19" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D34" s="20">
         <v>43609</v>
@@ -5898,16 +6067,16 @@
         <v/>
       </c>
       <c r="K34" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L34" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L34" s="19" t="s">
+      <c r="M34" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M34" s="19" t="s">
+      <c r="N34" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N34" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O34" s="20">
         <v>43972</v>
@@ -5956,7 +6125,7 @@
         <v>2031</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D35" s="20">
         <v>43617</v>
@@ -5979,16 +6148,16 @@
         <v/>
       </c>
       <c r="K35" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L35" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L35" s="19" t="s">
+      <c r="M35" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M35" s="19" t="s">
+      <c r="N35" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N35" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O35" s="20">
         <v>44320</v>
@@ -6037,7 +6206,7 @@
         <v>2032</v>
       </c>
       <c r="C36" s="19" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D36" s="20">
         <v>43622</v>
@@ -6060,16 +6229,16 @@
         <v/>
       </c>
       <c r="K36" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L36" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L36" s="19" t="s">
+      <c r="M36" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M36" s="19" t="s">
+      <c r="N36" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N36" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O36" s="20">
         <v>44060</v>
@@ -6118,7 +6287,7 @@
         <v>2033</v>
       </c>
       <c r="C37" s="35" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D37" s="36">
         <v>43621</v>
@@ -6143,16 +6312,16 @@
         <v>8.8732933848889653E-2</v>
       </c>
       <c r="K37" s="38" t="s">
+        <v>44</v>
+      </c>
+      <c r="L37" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="L37" s="35" t="s">
+      <c r="M37" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="M37" s="35" t="s">
-        <v>47</v>
-      </c>
       <c r="N37" s="35" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O37" s="36"/>
       <c r="P37" s="36"/>
@@ -6180,7 +6349,7 @@
         <v>0</v>
       </c>
       <c r="W37" s="35" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="X37" s="35"/>
       <c r="Y37" s="59">
@@ -6201,7 +6370,7 @@
         <v>2034</v>
       </c>
       <c r="C38" s="28" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D38" s="30">
         <v>43628</v>
@@ -6227,16 +6396,16 @@
         <v>2.7270109592942168E-2</v>
       </c>
       <c r="K38" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="L38" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="L38" s="28" t="s">
+      <c r="M38" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="M38" s="28" t="s">
-        <v>47</v>
-      </c>
       <c r="N38" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O38" s="30"/>
       <c r="P38" s="30"/>
@@ -6265,7 +6434,7 @@
       </c>
       <c r="W38" s="28"/>
       <c r="X38" s="28" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Y38" s="41">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -6285,7 +6454,7 @@
         <v>2035</v>
       </c>
       <c r="C39" s="19" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D39" s="20">
         <v>43629</v>
@@ -6308,16 +6477,16 @@
         <v/>
       </c>
       <c r="K39" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L39" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L39" s="19" t="s">
+      <c r="M39" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M39" s="19" t="s">
+      <c r="N39" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N39" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O39" s="20">
         <v>45456</v>
@@ -6366,7 +6535,7 @@
         <v>2036</v>
       </c>
       <c r="C40" s="19" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D40" s="20">
         <v>43777</v>
@@ -6389,16 +6558,16 @@
         <v/>
       </c>
       <c r="K40" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L40" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L40" s="19" t="s">
+      <c r="M40" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M40" s="19" t="s">
+      <c r="N40" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N40" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O40" s="20">
         <v>44581</v>
@@ -6447,7 +6616,7 @@
         <v>2037</v>
       </c>
       <c r="C41" s="19" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D41" s="20">
         <v>43784</v>
@@ -6470,16 +6639,16 @@
         <v/>
       </c>
       <c r="K41" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="L41" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="L41" s="19" t="s">
+      <c r="M41" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="M41" s="19" t="s">
+      <c r="N41" s="19" t="s">
         <v>47</v>
-      </c>
-      <c r="N41" s="19" t="s">
-        <v>48</v>
       </c>
       <c r="O41" s="20">
         <v>45225</v>
@@ -6528,7 +6697,7 @@
         <v>2038</v>
       </c>
       <c r="C42" s="35" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D42" s="36">
         <v>43798</v>
@@ -6555,16 +6724,16 @@
         <v>0.40476543842843071</v>
       </c>
       <c r="K42" s="38" t="s">
+        <v>95</v>
+      </c>
+      <c r="L42" s="35" t="s">
+        <v>58</v>
+      </c>
+      <c r="M42" s="35" t="s">
         <v>96</v>
       </c>
-      <c r="L42" s="35" t="s">
-        <v>59</v>
-      </c>
-      <c r="M42" s="35" t="s">
-        <v>97</v>
-      </c>
       <c r="N42" s="35" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="O42" s="36"/>
       <c r="P42" s="36"/>
@@ -6611,7 +6780,7 @@
         <v>2040</v>
       </c>
       <c r="C43" s="19" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D43" s="20">
         <v>44599</v>
@@ -6635,16 +6804,16 @@
         <v/>
       </c>
       <c r="K43" s="19" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L43" s="19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M43" s="19" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N43" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="O43" s="20">
         <v>44974</v>
@@ -6675,7 +6844,7 @@
       </c>
       <c r="W43" s="28"/>
       <c r="X43" s="29" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Y43" s="27">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -6695,7 +6864,7 @@
         <v>2041</v>
       </c>
       <c r="C44" s="28" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D44" s="30">
         <v>44553</v>
@@ -6722,16 +6891,16 @@
         <v>0.14317612367689922</v>
       </c>
       <c r="K44" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="L44" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="M44" s="28" t="s">
         <v>96</v>
       </c>
-      <c r="L44" s="28" t="s">
-        <v>59</v>
-      </c>
-      <c r="M44" s="28" t="s">
-        <v>97</v>
-      </c>
       <c r="N44" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O44" s="30"/>
       <c r="P44" s="41"/>
@@ -6778,7 +6947,7 @@
         <v>2042</v>
       </c>
       <c r="C45" s="28" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D45" s="30">
         <v>44709</v>
@@ -6805,16 +6974,16 @@
         <v>0.45354657164389256</v>
       </c>
       <c r="K45" s="32" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L45" s="28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M45" s="28" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N45" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O45" s="30"/>
       <c r="P45" s="41"/>
@@ -6843,7 +7012,7 @@
       </c>
       <c r="W45" s="28"/>
       <c r="X45" s="28" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Y45" s="41">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -6863,7 +7032,7 @@
         <v>2043</v>
       </c>
       <c r="C46" s="19" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D46" s="20">
         <v>44708</v>
@@ -6887,16 +7056,16 @@
         <v/>
       </c>
       <c r="K46" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="L46" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="M46" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="L46" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="M46" s="19" t="s">
-        <v>97</v>
-      </c>
       <c r="N46" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="O46" s="20">
         <v>45198</v>
@@ -6945,7 +7114,7 @@
         <v>2044</v>
       </c>
       <c r="C47" s="19" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D47" s="20">
         <v>44979</v>
@@ -6969,16 +7138,16 @@
         <v/>
       </c>
       <c r="K47" s="32" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L47" s="19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M47" s="19" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N47" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="O47" s="20">
         <v>45164</v>
@@ -7027,7 +7196,7 @@
         <v>2045</v>
       </c>
       <c r="C48" s="19" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D48" s="20">
         <v>45237</v>
@@ -7051,16 +7220,16 @@
         <v/>
       </c>
       <c r="K48" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="L48" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="M48" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="L48" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="M48" s="19" t="s">
-        <v>97</v>
-      </c>
       <c r="N48" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="O48" s="20">
         <v>45401</v>
@@ -7109,7 +7278,7 @@
         <v>2046</v>
       </c>
       <c r="C49" s="19" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D49" s="20">
         <v>45244</v>
@@ -7133,16 +7302,16 @@
         <v/>
       </c>
       <c r="K49" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="L49" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="M49" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="L49" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="M49" s="19" t="s">
-        <v>97</v>
-      </c>
       <c r="N49" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="O49" s="20">
         <v>45499</v>
@@ -7191,7 +7360,7 @@
         <v>2047</v>
       </c>
       <c r="C50" s="19" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D50" s="20">
         <v>45254</v>
@@ -7215,16 +7384,16 @@
         <v/>
       </c>
       <c r="K50" s="32" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L50" s="19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M50" s="19" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N50" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="O50" s="20">
         <v>45589</v>
@@ -7255,7 +7424,7 @@
       </c>
       <c r="W50" s="28"/>
       <c r="X50" s="29" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Y50" s="27">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -7275,7 +7444,7 @@
         <v>2048</v>
       </c>
       <c r="C51" s="28" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D51" s="30">
         <v>45258</v>
@@ -7301,16 +7470,16 @@
         <v>0.27130295109789371</v>
       </c>
       <c r="K51" s="32" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L51" s="28" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="M51" s="28" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N51" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O51" s="30"/>
       <c r="P51" s="41">
@@ -7342,7 +7511,7 @@
       </c>
       <c r="W51" s="28"/>
       <c r="X51" s="28" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="Y51" s="41">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -7362,7 +7531,7 @@
         <v>2049</v>
       </c>
       <c r="C52" s="19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D52" s="20">
         <v>45258</v>
@@ -7386,16 +7555,16 @@
         <v/>
       </c>
       <c r="K52" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="L52" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="M52" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="L52" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="M52" s="19" t="s">
-        <v>97</v>
-      </c>
       <c r="N52" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="O52" s="20">
         <v>45737</v>
@@ -7444,7 +7613,7 @@
         <v>2050</v>
       </c>
       <c r="C53" s="19" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D53" s="20">
         <v>45282</v>
@@ -7468,16 +7637,16 @@
         <v/>
       </c>
       <c r="K53" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="L53" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="M53" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="L53" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="M53" s="19" t="s">
-        <v>97</v>
-      </c>
       <c r="N53" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="O53" s="20">
         <v>45615</v>
@@ -7526,7 +7695,7 @@
         <v>2051</v>
       </c>
       <c r="C54" s="19" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D54" s="20">
         <v>45287</v>
@@ -7550,16 +7719,16 @@
         <v/>
       </c>
       <c r="K54" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="L54" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="M54" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="L54" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="M54" s="19" t="s">
-        <v>97</v>
-      </c>
       <c r="N54" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="O54" s="20">
         <v>45733</v>
@@ -7608,7 +7777,7 @@
         <v>2053</v>
       </c>
       <c r="C55" s="19" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D55" s="20">
         <v>45366</v>
@@ -7632,16 +7801,16 @@
         <v/>
       </c>
       <c r="K55" s="32" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L55" s="19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M55" s="19" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N55" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="O55" s="20">
         <v>45684</v>
@@ -7672,7 +7841,7 @@
       </c>
       <c r="W55" s="28"/>
       <c r="X55" s="29" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="Y55" s="27">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -7692,7 +7861,7 @@
         <v>2054</v>
       </c>
       <c r="C56" s="19" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D56" s="20">
         <v>45366</v>
@@ -7716,16 +7885,16 @@
         <v/>
       </c>
       <c r="K56" s="32" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L56" s="19" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M56" s="19" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N56" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="O56" s="20">
         <v>45489</v>
@@ -7756,7 +7925,7 @@
       </c>
       <c r="W56" s="28"/>
       <c r="X56" s="29" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="Y56" s="27">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -7776,7 +7945,7 @@
         <v>2055</v>
       </c>
       <c r="C57" s="28" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D57" s="30">
         <v>45385</v>
@@ -7802,16 +7971,16 @@
         <v>0.39252209720988157</v>
       </c>
       <c r="K57" s="32" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L57" s="28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M57" s="28" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N57" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O57" s="30"/>
       <c r="P57" s="41"/>
@@ -7840,7 +8009,7 @@
       </c>
       <c r="W57" s="28"/>
       <c r="X57" s="28" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="Y57" s="41">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -7860,7 +8029,7 @@
         <v>2056</v>
       </c>
       <c r="C58" s="28" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D58" s="30">
         <v>45470</v>
@@ -7886,16 +8055,16 @@
         <v>0.39936201917436892</v>
       </c>
       <c r="K58" s="32" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L58" s="28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M58" s="28" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N58" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O58" s="30"/>
       <c r="P58" s="41"/>
@@ -7924,7 +8093,7 @@
       </c>
       <c r="W58" s="28"/>
       <c r="X58" s="28" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Y58" s="41">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -7944,7 +8113,7 @@
         <v>2057</v>
       </c>
       <c r="C59" s="28" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D59" s="30">
         <v>45561</v>
@@ -7970,16 +8139,16 @@
         <v>0.34769933552284504</v>
       </c>
       <c r="K59" s="32" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L59" s="28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M59" s="28" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N59" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O59" s="30"/>
       <c r="P59" s="41"/>
@@ -8008,7 +8177,7 @@
       </c>
       <c r="W59" s="28"/>
       <c r="X59" s="28" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="Y59" s="41">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -8028,7 +8197,7 @@
         <v>2058</v>
       </c>
       <c r="C60" s="28" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D60" s="30">
         <v>45714</v>
@@ -8054,16 +8223,16 @@
         <v>0.39529999999999998</v>
       </c>
       <c r="K60" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="L60" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="M60" s="28" t="s">
         <v>96</v>
       </c>
-      <c r="L60" s="28" t="s">
-        <v>59</v>
-      </c>
-      <c r="M60" s="28" t="s">
-        <v>97</v>
-      </c>
       <c r="N60" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O60" s="30"/>
       <c r="P60" s="41"/>
@@ -8110,7 +8279,7 @@
         <v>2059</v>
       </c>
       <c r="C61" s="28" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D61" s="30">
         <v>45709</v>
@@ -8136,16 +8305,16 @@
         <v>0.36329999999999996</v>
       </c>
       <c r="K61" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="L61" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="M61" s="28" t="s">
         <v>96</v>
       </c>
-      <c r="L61" s="28" t="s">
-        <v>59</v>
-      </c>
-      <c r="M61" s="28" t="s">
-        <v>97</v>
-      </c>
       <c r="N61" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O61" s="30"/>
       <c r="P61" s="41"/>
@@ -8192,7 +8361,7 @@
         <v>2060</v>
       </c>
       <c r="C62" s="28" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D62" s="30">
         <v>45713</v>
@@ -8218,16 +8387,16 @@
         <v>0.24110033447057799</v>
       </c>
       <c r="K62" s="32" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L62" s="28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M62" s="28" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N62" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O62" s="30"/>
       <c r="P62" s="41"/>
@@ -8256,7 +8425,7 @@
       </c>
       <c r="W62" s="28"/>
       <c r="X62" s="28" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y62" s="41">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -8276,7 +8445,7 @@
         <v>2061</v>
       </c>
       <c r="C63" s="28" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D63" s="30">
         <v>45742</v>
@@ -8302,16 +8471,16 @@
         <v>0.42918032786885246</v>
       </c>
       <c r="K63" s="32" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L63" s="28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M63" s="28" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N63" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O63" s="30"/>
       <c r="P63" s="41"/>
@@ -8340,7 +8509,7 @@
       </c>
       <c r="W63" s="28"/>
       <c r="X63" s="28" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Y63" s="41">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -8360,7 +8529,7 @@
         <v>2062</v>
       </c>
       <c r="C64" s="28" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D64" s="30">
         <v>45791</v>
@@ -8386,16 +8555,16 @@
         <v>0.33166343079743738</v>
       </c>
       <c r="K64" s="32" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L64" s="28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M64" s="28" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N64" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O64" s="30"/>
       <c r="P64" s="41"/>
@@ -8424,7 +8593,7 @@
       </c>
       <c r="W64" s="28"/>
       <c r="X64" s="28" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y64" s="41">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -8444,7 +8613,7 @@
         <v>2063</v>
       </c>
       <c r="C65" s="28" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D65" s="30">
         <v>45853</v>
@@ -8470,16 +8639,16 @@
         <v>7.9338897894184746E-2</v>
       </c>
       <c r="K65" s="32" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L65" s="28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M65" s="28" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="N65" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O65" s="30"/>
       <c r="P65" s="41"/>
@@ -8508,7 +8677,7 @@
       </c>
       <c r="W65" s="28"/>
       <c r="X65" s="28" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="Y65" s="41">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -8528,7 +8697,7 @@
         <v>2064</v>
       </c>
       <c r="C66" s="28" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D66" s="30">
         <v>45860</v>
@@ -8554,16 +8723,16 @@
         <v>0.3797551326169909</v>
       </c>
       <c r="K66" s="32" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L66" s="28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M66" s="28" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N66" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O66" s="30"/>
       <c r="P66" s="41"/>
@@ -8592,7 +8761,7 @@
       </c>
       <c r="W66" s="28"/>
       <c r="X66" s="28" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Y66" s="41">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -8612,7 +8781,7 @@
         <v>2065</v>
       </c>
       <c r="C67" s="28" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D67" s="30">
         <v>45961</v>
@@ -8638,16 +8807,16 @@
         <v>0.39844226635420765</v>
       </c>
       <c r="K67" s="32" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L67" s="28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M67" s="28" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N67" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O67" s="30"/>
       <c r="P67" s="41"/>
@@ -8676,7 +8845,7 @@
       </c>
       <c r="W67" s="28"/>
       <c r="X67" s="28" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y67" s="41">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -8696,7 +8865,7 @@
         <v>2066</v>
       </c>
       <c r="C68" s="28" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D68" s="30">
         <v>46001</v>
@@ -8722,16 +8891,16 @@
         <v>0.35695481934394546</v>
       </c>
       <c r="K68" s="32" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L68" s="28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M68" s="28" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="N68" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O68" s="30"/>
       <c r="P68" s="41"/>
@@ -8760,7 +8929,7 @@
       </c>
       <c r="W68" s="28"/>
       <c r="X68" s="28" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="Y68" s="41">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -8780,7 +8949,7 @@
         <v>2067</v>
       </c>
       <c r="C69" s="28" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D69" s="30">
         <v>46009</v>
@@ -8806,16 +8975,16 @@
         <v>0.22137932305528329</v>
       </c>
       <c r="K69" s="32" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L69" s="28" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M69" s="28" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="N69" s="28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="O69" s="30"/>
       <c r="P69" s="41"/>
@@ -8844,7 +9013,7 @@
       </c>
       <c r="W69" s="28"/>
       <c r="X69" s="28" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="Y69" s="41">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Activos",IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Francés",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],DATE(YEAR(TODAY()),1,1),"m"),0),0)</f>
@@ -8882,10 +9051,10 @@
   <sheetData>
     <row r="2" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.2">
@@ -8893,7 +9062,7 @@
         <v>2201</v>
       </c>
       <c r="C3" s="28" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.2">
@@ -8901,7 +9070,7 @@
         <v>2202</v>
       </c>
       <c r="C4" s="28" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.2">
@@ -8909,7 +9078,7 @@
         <v>2203</v>
       </c>
       <c r="C5" s="28" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.2">
@@ -8917,7 +9086,7 @@
         <v>2204</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.2">
@@ -8925,7 +9094,7 @@
         <v>2205</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.2">
@@ -8933,7 +9102,7 @@
         <v>2206</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -8963,7 +9132,7 @@
   <sheetData>
     <row r="2" spans="2:16" ht="19" x14ac:dyDescent="0.25">
       <c r="B2" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C2" s="14"/>
       <c r="D2" s="14"/>
@@ -8981,49 +9150,49 @@
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B3" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="D3" s="5" t="s">
+      <c r="E3" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>152</v>
-      </c>
       <c r="G3" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>1</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="2:16" x14ac:dyDescent="0.2">
@@ -9056,7 +9225,7 @@
         <v>45448</v>
       </c>
       <c r="J4" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K4" s="4">
         <v>0.02</v>
@@ -9111,7 +9280,7 @@
         <v>45448</v>
       </c>
       <c r="J5" s="51" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K5" s="60">
         <v>0.02</v>
@@ -9166,7 +9335,7 @@
         <v>45448</v>
       </c>
       <c r="J6" s="20" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K6" s="60">
         <v>0.02</v>
@@ -9221,7 +9390,7 @@
         <v>45448</v>
       </c>
       <c r="J7" s="51" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K7" s="60">
         <v>0.02</v>
@@ -9276,7 +9445,7 @@
         <v>45470</v>
       </c>
       <c r="J8" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K8" s="4">
         <v>0.02</v>
@@ -9331,7 +9500,7 @@
         <v>45561</v>
       </c>
       <c r="J9" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K9" s="4">
         <v>0.02</v>
@@ -9386,7 +9555,7 @@
         <v>45593</v>
       </c>
       <c r="J10" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K10" s="4">
         <v>0.02</v>
@@ -9441,7 +9610,7 @@
         <v>45587</v>
       </c>
       <c r="J11" s="20" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K11" s="60">
         <v>0.02</v>
@@ -9496,7 +9665,7 @@
         <v>45587</v>
       </c>
       <c r="J12" s="20" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K12" s="60">
         <v>0.02</v>
@@ -9551,7 +9720,7 @@
         <v>45587</v>
       </c>
       <c r="J13" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K13" s="4">
         <v>0.02</v>
@@ -9606,7 +9775,7 @@
         <v>45742</v>
       </c>
       <c r="J14" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K14" s="4">
         <v>0.02</v>
@@ -9661,7 +9830,7 @@
         <v>45742</v>
       </c>
       <c r="J15" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K15" s="4">
         <v>0.02</v>
@@ -9716,7 +9885,7 @@
         <v>45742</v>
       </c>
       <c r="J16" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K16" s="4">
         <v>0.02</v>
@@ -9771,7 +9940,7 @@
         <v>45742</v>
       </c>
       <c r="J17" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K17" s="4">
         <v>0.02</v>
@@ -9826,7 +9995,7 @@
         <v>45742</v>
       </c>
       <c r="J18" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K18" s="4">
         <v>0.02</v>
@@ -9881,7 +10050,7 @@
         <v>45853</v>
       </c>
       <c r="J19" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K19" s="4">
         <v>0.02</v>
@@ -9936,7 +10105,7 @@
         <v>45860</v>
       </c>
       <c r="J20" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K20" s="4">
         <v>0.02</v>
@@ -9991,7 +10160,7 @@
         <v>45860</v>
       </c>
       <c r="J21" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K21" s="4">
         <v>0.02</v>
@@ -10046,7 +10215,7 @@
         <v>45891</v>
       </c>
       <c r="J22" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K22" s="4">
         <v>0.02</v>
@@ -10101,7 +10270,7 @@
         <v>45891</v>
       </c>
       <c r="J23" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K23" s="4">
         <v>0.02</v>
@@ -10156,7 +10325,7 @@
         <v>45891</v>
       </c>
       <c r="J24" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K24" s="4">
         <v>0.02</v>
@@ -10211,7 +10380,7 @@
         <v>45891</v>
       </c>
       <c r="J25" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K25" s="4">
         <v>0.02</v>
@@ -10266,7 +10435,7 @@
         <v>45891</v>
       </c>
       <c r="J26" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K26" s="4">
         <v>0.02</v>
@@ -10321,7 +10490,7 @@
         <v>45961</v>
       </c>
       <c r="J27" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K27" s="4">
         <v>0.02</v>
@@ -10376,7 +10545,7 @@
         <v>45961</v>
       </c>
       <c r="J28" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K28" s="4">
         <v>0.02</v>
@@ -10431,7 +10600,7 @@
         <v>45971</v>
       </c>
       <c r="J29" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K29" s="4">
         <v>0.02</v>
@@ -10490,7 +10659,7 @@
         <v>45971</v>
       </c>
       <c r="J30" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K30" s="4">
         <v>0.02</v>
@@ -10545,7 +10714,7 @@
         <v>45971</v>
       </c>
       <c r="J31" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K31" s="4">
         <v>0.02</v>
@@ -10600,7 +10769,7 @@
         <v>46001</v>
       </c>
       <c r="J32" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K32" s="4">
         <v>0.02</v>
@@ -10657,7 +10826,7 @@
         <v>46001</v>
       </c>
       <c r="J33" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K33" s="4">
         <v>0.02</v>
@@ -10712,7 +10881,7 @@
         <v>46009</v>
       </c>
       <c r="J34" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K34" s="4">
         <v>0.02</v>
@@ -10769,7 +10938,7 @@
         <v>46009</v>
       </c>
       <c r="J35" s="30" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K35" s="4">
         <v>0</v>
@@ -10804,7 +10973,7 @@
     </row>
     <row r="37" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B37" s="57" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C37" s="57"/>
       <c r="D37" s="57"/>
@@ -10817,7 +10986,7 @@
     </row>
     <row r="38" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B38" s="57" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C38" s="57"/>
       <c r="D38" s="57"/>
@@ -10834,7 +11003,7 @@
     </row>
     <row r="39" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B39" s="57" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C39" s="57"/>
       <c r="D39" s="57"/>

</xml_diff>

<commit_message>
Hemos implementado algunos tests y estamos depurandolos. Última versión con amortizaciones parciales en medio de un préstamo. Abordamos el cambio de que una AP cree un nuevo préstamo
</commit_message>
<xml_diff>
--- a/documentación/Cálculos aplicación.xlsx
+++ b/documentación/Cálculos aplicación.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/narcismagrinabalcells/Dropbox/1 - OFICINA/1-PROMOCIMA/02-CAPITAL PRIVADO/30 - Desarrollo/Préstamos/Claude Pro/promocima/documentación/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD5C8CC6-27F6-5949-A567-B2F49F561007}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{009542C0-7525-F644-A79A-B3E72EDC6200}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30980" yWindow="1860" windowWidth="26260" windowHeight="19700" activeTab="1" xr2:uid="{7DA0983C-EA6B-584E-90AC-C5A5D261DBFA}"/>
+    <workbookView xWindow="6120" yWindow="2760" windowWidth="26260" windowHeight="19700" activeTab="1" xr2:uid="{7DA0983C-EA6B-584E-90AC-C5A5D261DBFA}"/>
   </bookViews>
   <sheets>
     <sheet name="Cálculo pagos" sheetId="1" r:id="rId1"/>
@@ -3117,7 +3117,7 @@
       </c>
       <c r="O17" s="56">
         <f ca="1">(SUMIFS(T_Prestamos[Duración],T_Prestamos[Situación],"Activos")+SUMIFS(T_Prestamos[Duración],T_Prestamos[Situación],"Judicializados"))/(COUNTIFS(T_Prestamos[Situación],"Activos")+COUNTIFS(T_Prestamos[Situación],"Judicializados"))</f>
-        <v>1342.7692307692307</v>
+        <v>1343.7692307692307</v>
       </c>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.2">
@@ -3191,7 +3191,7 @@
       </c>
       <c r="O19" s="11">
         <f ca="1">SUMIFS(T_Prestamos[Duración],T_Prestamos[Situación],"Activos")/COUNTIFS(T_Prestamos[Situación],"Activos")</f>
-        <v>1120.0454545454545</v>
+        <v>1121.0454545454545</v>
       </c>
     </row>
     <row r="20" spans="2:15" x14ac:dyDescent="0.2">
@@ -3228,7 +3228,7 @@
       </c>
       <c r="O20" s="11">
         <f ca="1">SUMIFS(T_Prestamos[Duración],T_Prestamos[Situación],"Judicializados")/COUNTIFS(T_Prestamos[Situación],"Judicializados")</f>
-        <v>2567.75</v>
+        <v>2568.75</v>
       </c>
     </row>
     <row r="21" spans="2:15" x14ac:dyDescent="0.2">
@@ -3278,7 +3278,7 @@
         <v>176</v>
       </c>
       <c r="C23" s="11">
-        <f>C22/C21</f>
+        <f>C22/(C21+C22)</f>
         <v>0</v>
       </c>
       <c r="E23" t="s">
@@ -3945,7 +3945,7 @@
       <c r="P8" s="30"/>
       <c r="Q8" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>3056</v>
+        <v>3057</v>
       </c>
       <c r="R8" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -4115,7 +4115,7 @@
       </c>
       <c r="R10" s="24">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="S10" s="25">
         <f>IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",0,IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Americano",T_Prestamos[[#This Row],[Importe]],T_Prestamos[[#This Row],[Importe]]+CUMPRINC(G10/12,E10*12,F10,1,R10,0)))</f>
@@ -4196,7 +4196,7 @@
       </c>
       <c r="R11" s="24">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="S11" s="25">
         <f>IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",0,IF(T_Prestamos[[#This Row],[Tipo préstamo]]="Americano",T_Prestamos[[#This Row],[Importe]],T_Prestamos[[#This Row],[Importe]]+CUMPRINC(G11/12,E11*12,F11,1,R11,0)))</f>
@@ -4598,7 +4598,7 @@
       <c r="P16" s="30"/>
       <c r="Q16" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>2928</v>
+        <v>2929</v>
       </c>
       <c r="R16" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -4936,7 +4936,7 @@
       <c r="P20" s="30"/>
       <c r="Q20" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>2817</v>
+        <v>2818</v>
       </c>
       <c r="R20" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -5181,7 +5181,7 @@
       <c r="P23" s="36"/>
       <c r="Q23" s="37">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>2777</v>
+        <v>2778</v>
       </c>
       <c r="R23" s="37">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -5345,7 +5345,7 @@
       <c r="P25" s="36"/>
       <c r="Q25" s="37">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>2721</v>
+        <v>2722</v>
       </c>
       <c r="R25" s="37">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -5755,7 +5755,7 @@
       <c r="P30" s="30"/>
       <c r="Q30" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>2572</v>
+        <v>2573</v>
       </c>
       <c r="R30" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -5920,7 +5920,7 @@
       <c r="P32" s="30"/>
       <c r="Q32" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>2553</v>
+        <v>2554</v>
       </c>
       <c r="R32" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -6327,7 +6327,7 @@
       <c r="P37" s="36"/>
       <c r="Q37" s="37">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>2475</v>
+        <v>2476</v>
       </c>
       <c r="R37" s="37">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -6411,7 +6411,7 @@
       <c r="P38" s="30"/>
       <c r="Q38" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>2468</v>
+        <v>2469</v>
       </c>
       <c r="R38" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -6739,7 +6739,7 @@
       <c r="P42" s="36"/>
       <c r="Q42" s="37">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>2298</v>
+        <v>2299</v>
       </c>
       <c r="R42" s="37">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -6906,7 +6906,7 @@
       <c r="P44" s="41"/>
       <c r="Q44" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>1543</v>
+        <v>1544</v>
       </c>
       <c r="R44" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -6989,7 +6989,7 @@
       <c r="P45" s="41"/>
       <c r="Q45" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>1387</v>
+        <v>1388</v>
       </c>
       <c r="R45" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -7488,7 +7488,7 @@
       </c>
       <c r="Q51" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="R51" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -7986,7 +7986,7 @@
       <c r="P57" s="41"/>
       <c r="Q57" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="R57" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -8070,7 +8070,7 @@
       <c r="P58" s="41"/>
       <c r="Q58" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="R58" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -8154,7 +8154,7 @@
       <c r="P59" s="41"/>
       <c r="Q59" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="R59" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -8238,7 +8238,7 @@
       <c r="P60" s="41"/>
       <c r="Q60" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="R60" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -8320,7 +8320,7 @@
       <c r="P61" s="41"/>
       <c r="Q61" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="R61" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -8402,7 +8402,7 @@
       <c r="P62" s="41"/>
       <c r="Q62" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="R62" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -8486,7 +8486,7 @@
       <c r="P63" s="41"/>
       <c r="Q63" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="R63" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -8570,7 +8570,7 @@
       <c r="P64" s="41"/>
       <c r="Q64" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="R64" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -8654,7 +8654,7 @@
       <c r="P65" s="41"/>
       <c r="Q65" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="R65" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -8738,7 +8738,7 @@
       <c r="P66" s="41"/>
       <c r="Q66" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="R66" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -8822,7 +8822,7 @@
       <c r="P67" s="41"/>
       <c r="Q67" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="R67" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -8906,7 +8906,7 @@
       <c r="P68" s="41"/>
       <c r="Q68" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="R68" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>
@@ -8990,7 +8990,7 @@
       <c r="P69" s="41"/>
       <c r="Q69" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelados",T_Prestamos[[#This Row],[Fecha cancelación]],TODAY())-T_Prestamos[[#This Row],[firma préstamo]]</f>
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="R69" s="31">
         <f ca="1">IF(T_Prestamos[[#This Row],[Situación]]="Cancelada","",DATEDIF(T_Prestamos[[#This Row],[firma préstamo]],TODAY(),"m"))</f>

</xml_diff>